<commit_message>
Add RAG pipeline, move tools to services, update prototype
Introduce rag_data.json, FAISS index builder, RagService; relocate vinschool_tools under services; add index.html entry and prototype-data.js; refresh mockdata and prototype shell.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/AI20K_VinSchoolOne_Mockdata.xlsx
+++ b/AI20K_VinSchoolOne_Mockdata.xlsx
@@ -13,6 +13,7 @@
     <sheet state="visible" name="Thời khoá biểu" sheetId="8" r:id="rId12"/>
     <sheet state="visible" name="Nhận xét" sheetId="9" r:id="rId13"/>
     <sheet state="visible" name="Kết quả học tập" sheetId="10" r:id="rId14"/>
+    <sheet state="visible" name="Thông báo" sheetId="11" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr/>
@@ -20,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="872" uniqueCount="469">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="953" uniqueCount="539">
   <si>
     <t>Họ tên</t>
   </si>
@@ -1450,6 +1451,216 @@
   </si>
   <si>
     <t>Thể hiện được vai trò trưởng nhóm trong các hoạt động lắp ráp, tạo hình.</t>
+  </si>
+  <si>
+    <t>STT</t>
+  </si>
+  <si>
+    <t>Loại thông báo</t>
+  </si>
+  <si>
+    <t>Tiêu đề</t>
+  </si>
+  <si>
+    <t>Nội dung tóm tắt</t>
+  </si>
+  <si>
+    <t>Đối tượng nhận</t>
+  </si>
+  <si>
+    <t>Ngày sự kiện</t>
+  </si>
+  <si>
+    <t>Hạn chót (Deadline)</t>
+  </si>
+  <si>
+    <t>Trạng thái hiển thị nút</t>
+  </si>
+  <si>
+    <t>Khảo sát</t>
+  </si>
+  <si>
+    <t>Khảo sát mức độ hài lòng &amp; nhu cầu sử dụng Vinschool One</t>
+  </si>
+  <si>
+    <t>Nhằm nâng cao chất lượng phối hợp dạy – học và dịch vụ số cho học sinh. Khảo sát kéo dài 5-7 phút phục vụ mục đích cải tiến dịch vụ.</t>
+  </si>
+  <si>
+    <t>PHHS Tiểu học – THCS – THPT</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>Không ghi rõ</t>
+  </si>
+  <si>
+    <t>Thực hiện khảo sát</t>
+  </si>
+  <si>
+    <t>Hoạt động ngoại khóa</t>
+  </si>
+  <si>
+    <t>Khảo sát ý kiến PHHS về việc HS tham gia hoạt động ngoại khóa "Bảo tàng đường Hồ Chí Minh"</t>
+  </si>
+  <si>
+    <t>Nhằm mang đến trải nghiệm học tập môn Lịch sử - Địa lí, giúp các con tìm hiểu chặng đường lịch sử hào hùng qua hiện vật và câu chuyện lịch sử.</t>
+  </si>
+  <si>
+    <t>PHHS Khối 5 (Vinschool Times City)</t>
+  </si>
+  <si>
+    <t>Trước 08/04/2026</t>
+  </si>
+  <si>
+    <t>Xem câu trả lời</t>
+  </si>
+  <si>
+    <t>Trải nghiệm học tập</t>
+  </si>
+  <si>
+    <t>Khảo sát PHHS về việc tham gia hoạt động trải nghiệm xem phim khối 5</t>
+  </si>
+  <si>
+    <t>Trải nghiệm thực tế môn ESL (Unit 8: Entertainment). Học sinh xem phim "Super Mario Galaxy" để tìm hiểu lịch sử rạp chiếu phim và trò chơi điện tử.</t>
+  </si>
+  <si>
+    <t>Cập nhật khảo sát</t>
+  </si>
+  <si>
+    <t>Học vụ</t>
+  </si>
+  <si>
+    <t>Thông báo lịch thi Giữa học kỳ 2</t>
+  </si>
+  <si>
+    <t>Lịch thi chi tiết các môn Toán, Tiếng Việt, Tiếng Anh và các môn chuyên biệt. PH vui lòng nhắc con ôn tập theo đề cương.</t>
+  </si>
+  <si>
+    <t>Toàn học sinh</t>
+  </si>
+  <si>
+    <t>02/03 - 06/03</t>
+  </si>
+  <si>
+    <t>Xem chi tiết</t>
+  </si>
+  <si>
+    <t>Sự kiện</t>
+  </si>
+  <si>
+    <t>Ngày hội Thể thao Vinschool (Sports Day)</t>
+  </si>
+  <si>
+    <t>Sự kiện thể thao thường niên nhằm rèn luyện sức khỏe và tinh thần đồng đội. Yêu cầu HS mặc đồng phục thể thao và mang theo nước uống.</t>
+  </si>
+  <si>
+    <t>Khối Tiểu học</t>
+  </si>
+  <si>
+    <t>Đăng ký tham gia</t>
+  </si>
+  <si>
+    <t>Y tế</t>
+  </si>
+  <si>
+    <t>Khám sức khỏe định kỳ đợt 2</t>
+  </si>
+  <si>
+    <t>Nhà trường phối hợp với bệnh viện Vinmec tổ chức khám sức khỏe tổng quát (mắt, răng miệng, chiều cao, cân nặng) cho học sinh.</t>
+  </si>
+  <si>
+    <t>10/03 - 12/03</t>
+  </si>
+  <si>
+    <t>Xem kết quả</t>
+  </si>
+  <si>
+    <t>Chào mừng ngày Quốc tế Phụ nữ 8/3</t>
+  </si>
+  <si>
+    <t>Hoạt động làm thiệp và quà handmade dành tặng mẹ và cô giáo trong giờ trải nghiệm sáng tạo.</t>
+  </si>
+  <si>
+    <t>Đã đóng</t>
+  </si>
+  <si>
+    <t>Hội thảo</t>
+  </si>
+  <si>
+    <t>Hội thảo: Định hướng tư duy AI cho trẻ</t>
+  </si>
+  <si>
+    <t>Buổi chia sẻ từ các chuyên gia về cách tiếp cận công nghệ và trí tuệ nhân tạo an toàn, hiệu quả cho học sinh phổ thông.</t>
+  </si>
+  <si>
+    <t>PHHS toàn trường</t>
+  </si>
+  <si>
+    <t>Đăng ký ngay</t>
+  </si>
+  <si>
+    <t>Thông báo họp Phụ huynh giữa học kỳ 2</t>
+  </si>
+  <si>
+    <t>Họp tập trung để trao đổi về tình hình học tập, rèn luyện và định hướng các hoạt động trong giai đoạn cuối năm học.</t>
+  </si>
+  <si>
+    <t>Xác nhận tham dự</t>
+  </si>
+  <si>
+    <t>Tài chính</t>
+  </si>
+  <si>
+    <t>Thông báo học phí và các khoản phí tháng 4/2026</t>
+  </si>
+  <si>
+    <t>Nhà trường gửi thông báo thu học phí, tiền ăn và phí xe đưa đón tháng 4. PH vui lòng thanh toán đúng hạn.</t>
+  </si>
+  <si>
+    <t>Hạn 31/03</t>
+  </si>
+  <si>
+    <t>Thanh toán ngay</t>
+  </si>
+  <si>
+    <t>Ngoại khóa</t>
+  </si>
+  <si>
+    <t>Đăng ký câu lạc bộ ngoại khóa sau giờ học</t>
+  </si>
+  <si>
+    <t>Mở cổng đăng ký các CLB: Bóng rổ, Lập trình Python, Vẽ sáng tạo và Nhảy hiện đại cho học kỳ mới.</t>
+  </si>
+  <si>
+    <t>01/04 - 30/05</t>
+  </si>
+  <si>
+    <t>Đăng ký</t>
+  </si>
+  <si>
+    <t>Ngày hội Đọc sách (Book Fair 2026)</t>
+  </si>
+  <si>
+    <t>Hoạt động trao đổi sách, kể chuyện theo nhân vật và gian hàng sách ưu đãi từ các nhà xuất bản lớn.</t>
+  </si>
+  <si>
+    <t>Xem lịch trình</t>
+  </si>
+  <si>
+    <t>Đời sống</t>
+  </si>
+  <si>
+    <t>Cập nhật thực đơn tháng 4/2026</t>
+  </si>
+  <si>
+    <t>Danh sách thực đơn bữa sáng, bữa trưa và bữa xế đã được kiểm duyệt bởi chuyên gia dinh dưỡng.</t>
+  </si>
+  <si>
+    <t>01/04 - 30/04</t>
+  </si>
+  <si>
+    <t>Xem thực đơn</t>
   </si>
 </sst>
 </file>
@@ -1555,6 +1766,10 @@
 </file>
 
 <file path=xl/drawings/drawing10.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/drawings/drawing11.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
@@ -2054,6 +2269,386 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <cols>
+    <col customWidth="1" min="3" max="3" width="73.38"/>
+    <col customWidth="1" min="4" max="4" width="26.5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="s">
+        <v>469</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>470</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>471</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>473</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>474</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>475</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4">
+        <v>1.0</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>477</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>478</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>479</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>480</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>481</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>482</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>483</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4">
+        <v>2.0</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>484</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>485</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>486</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>487</v>
+      </c>
+      <c r="F3" s="8">
+        <v>46120.0</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>488</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4">
+        <v>3.0</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>490</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>491</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>492</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>487</v>
+      </c>
+      <c r="F4" s="8">
+        <v>46122.0</v>
+      </c>
+      <c r="G4" s="8">
+        <v>46121.0</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>493</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4">
+        <v>4.0</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>494</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>495</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>496</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>497</v>
+      </c>
+      <c r="F5" s="8">
+        <v>46072.0</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>498</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4">
+        <v>5.0</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>500</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>501</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>502</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>503</v>
+      </c>
+      <c r="F6" s="8">
+        <v>46078.0</v>
+      </c>
+      <c r="G6" s="8">
+        <v>46088.0</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4">
+        <v>6.0</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>505</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>506</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>507</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>497</v>
+      </c>
+      <c r="F7" s="8">
+        <v>46083.0</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>508</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4">
+        <v>7.0</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>500</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>510</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>511</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>503</v>
+      </c>
+      <c r="F8" s="8">
+        <v>46086.0</v>
+      </c>
+      <c r="G8" s="8">
+        <v>46089.0</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4">
+        <v>8.0</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>513</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>514</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>515</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>516</v>
+      </c>
+      <c r="F9" s="8">
+        <v>46090.0</v>
+      </c>
+      <c r="G9" s="8">
+        <v>46096.0</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>517</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4">
+        <v>9.0</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>494</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>518</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>519</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>516</v>
+      </c>
+      <c r="F10" s="8">
+        <v>46093.0</v>
+      </c>
+      <c r="G10" s="8">
+        <v>46102.0</v>
+      </c>
+      <c r="H10" s="4" t="s">
+        <v>520</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4">
+        <v>10.0</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>521</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>522</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>523</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>516</v>
+      </c>
+      <c r="F11" s="8">
+        <v>46099.0</v>
+      </c>
+      <c r="G11" s="4" t="s">
+        <v>524</v>
+      </c>
+      <c r="H11" s="4" t="s">
+        <v>525</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4">
+        <v>11.0</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>526</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>527</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>528</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>503</v>
+      </c>
+      <c r="F12" s="8">
+        <v>46104.0</v>
+      </c>
+      <c r="G12" s="4" t="s">
+        <v>529</v>
+      </c>
+      <c r="H12" s="4" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4">
+        <v>12.0</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>500</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>531</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>532</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>497</v>
+      </c>
+      <c r="F13" s="8">
+        <v>46107.0</v>
+      </c>
+      <c r="G13" s="8">
+        <v>46116.0</v>
+      </c>
+      <c r="H13" s="4" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4">
+        <v>13.0</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>534</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>535</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>536</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>516</v>
+      </c>
+      <c r="F14" s="8">
+        <v>46111.0</v>
+      </c>
+      <c r="G14" s="4" t="s">
+        <v>537</v>
+      </c>
+      <c r="H14" s="4" t="s">
+        <v>538</v>
+      </c>
+    </row>
+  </sheetData>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>

</xml_diff>